<commit_message>
evaluation of the bayensian model + plots
</commit_message>
<xml_diff>
--- a/seuils.xlsx
+++ b/seuils.xlsx
@@ -471,12 +471,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-3.03</t>
+          <t>-3.05</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.472</t>
+          <t>0.483</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -490,10 +490,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>6994</v>
+        <v>8112</v>
       </c>
       <c r="G2" t="n">
-        <v>3354</v>
+        <v>3092</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -502,12 +502,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.0056</t>
+          <t>0.0054</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>0.0041</t>
+          <t>0.0037</t>
         </is>
       </c>
     </row>
@@ -519,12 +519,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-1.04</t>
+          <t>-1.06</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.47</t>
+          <t>0.48</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -534,14 +534,14 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-0.31</t>
+          <t>-0.29</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>7127</v>
+        <v>8565</v>
       </c>
       <c r="G3" t="n">
-        <v>3348</v>
+        <v>3089</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -550,12 +550,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.0056</t>
+          <t>0.0052</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.004</t>
+          <t>0.0036</t>
         </is>
       </c>
     </row>
@@ -567,17 +567,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.93</t>
+          <t>0.92</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.469</t>
+          <t>0.48</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.19</t>
+          <t>0.16</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -586,10 +586,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>7054</v>
+        <v>8771</v>
       </c>
       <c r="G4" t="n">
-        <v>3180</v>
+        <v>3144</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -598,12 +598,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.0056</t>
+          <t>0.0051</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.0041</t>
+          <t>0.0036</t>
         </is>
       </c>
     </row>
@@ -615,29 +615,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3.11</t>
+          <t>3.09</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.473</t>
+          <t>0.482</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3.8</t>
+          <t>3.9</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>7253</v>
+        <v>8856</v>
       </c>
       <c r="G5" t="n">
-        <v>3301</v>
+        <v>3146</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -646,12 +646,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.0055</t>
+          <t>0.0051</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0.004</t>
+          <t>0.0036</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test of model_2 + reorganisation of the code
</commit_message>
<xml_diff>
--- a/seuils.xlsx
+++ b/seuils.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-3.05</t>
+          <t>-3.04</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -490,10 +490,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>8112</v>
+        <v>6527</v>
       </c>
       <c r="G2" t="n">
-        <v>3092</v>
+        <v>3070</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -502,12 +502,12 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.0054</t>
+          <t>0.006</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>0.0037</t>
+          <t>0.0042</t>
         </is>
       </c>
     </row>
@@ -519,12 +519,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-1.06</t>
+          <t>-1.05</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.48</t>
+          <t>0.484</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -534,14 +534,14 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-0.29</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>8565</v>
+        <v>6784</v>
       </c>
       <c r="G3" t="n">
-        <v>3089</v>
+        <v>3096</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -550,12 +550,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.0052</t>
+          <t>0.0058</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>0.0036</t>
+          <t>0.0041</t>
         </is>
       </c>
     </row>
@@ -567,17 +567,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.92</t>
+          <t>0.93</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.48</t>
+          <t>0.484</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -586,10 +586,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>8771</v>
+        <v>6990</v>
       </c>
       <c r="G4" t="n">
-        <v>3144</v>
+        <v>3063</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -598,12 +598,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.0051</t>
+          <t>0.0058</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.0036</t>
+          <t>0.0041</t>
         </is>
       </c>
     </row>
@@ -615,12 +615,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3.09</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.482</t>
+          <t>0.486</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -634,10 +634,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>8856</v>
+        <v>6951</v>
       </c>
       <c r="G5" t="n">
-        <v>3146</v>
+        <v>3119</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -646,12 +646,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.0051</t>
+          <t>0.0058</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0.0036</t>
+          <t>0.0041</t>
         </is>
       </c>
     </row>

</xml_diff>